<commit_message>
Keynote workbook: stacked-bar layout (Cards/Shipping per bar)
Add 'Stacked bars' tab: one row per bucket x vendor with Cards and
Shipping as the two stack columns, so Keynote renders shipping broken
out. Keep wide by-bucket tab for a grouped-stacked rebuild.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/keynote_standard_basket.xlsx
+++ b/output/keynote_standard_basket.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Chart data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All-in totals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Stacked bars" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Wide (by bucket)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -70,17 +69,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -447,59 +445,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Basket (cards)</t>
+          <t>Bar</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>CK cards</t>
+          <t>Cards</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>CK shipping</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>TCG cards</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>TCG shipping</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>MP cards</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>MP shipping</t>
+          <t>Shipping</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>0-5</t>
+          <t>0-5  Card Kingdom</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -508,116 +482,186 @@
       <c r="C2" s="3" t="n">
         <v>4.97</v>
       </c>
-      <c r="D2" s="3" t="n">
-        <v>9.470000000000001</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>8.59</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>3.96</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>5-20</t>
+          <t>0-5  TCGplayer</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>48.9</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>41.88</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>4.98</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>38.34</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>2.87</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>20-50</t>
+          <t>0-5  ManaPool</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>130.91</v>
+        <v>8.59</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>111.36</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>11.12</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>101.42</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>50-75</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>230.76</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>196.89</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>180.24</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>0</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>75-100</t>
+          <t>5-20  Card Kingdom</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>4.18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>5-20  TCGplayer</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>4.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>5-20  ManaPool</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>2.87</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>20-50  Card Kingdom</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>130.91</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>20-50  TCGplayer</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>111.36</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>11.12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>20-50  ManaPool</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>101.42</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>50-75  Card Kingdom</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>230.76</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>50-75  TCGplayer</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>196.89</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>50-75  ManaPool</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>180.24</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>75-100  Card Kingdom</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
         <v>317.09</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="3" t="n">
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>75-100  TCGplayer</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
         <v>270.23</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="C19" s="3" t="n">
         <v>29.76</v>
       </c>
-      <c r="F6" s="3" t="n">
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>75-100  ManaPool</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
         <v>247.83</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="C20" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -632,34 +676,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Basket (cards)</t>
+          <t>Basket</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Card Kingdom</t>
+          <t>CK cards</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>TCGplayer</t>
+          <t>CK ship</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>ManaPool</t>
+          <t>TCG cards</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>TCG ship</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>MP cards</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>MP ship</t>
         </is>
       </c>
     </row>
@@ -669,14 +731,23 @@
           <t>0-5</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
-        <v>16.34</v>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>12.55</v>
+      <c r="B2" s="3" t="n">
+        <v>11.37</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>8.59</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>3.96</v>
       </c>
     </row>
     <row r="3">
@@ -685,14 +756,23 @@
           <t>5-20</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
-        <v>53.08</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>46.86</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>41.21</v>
+      <c r="B3" s="3" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>2.87</v>
       </c>
     </row>
     <row r="4">
@@ -701,14 +781,23 @@
           <t>20-50</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>131.56</v>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>122.48</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>101.82</v>
+      <c r="B4" s="3" t="n">
+        <v>130.91</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>111.36</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>11.12</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>101.42</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="5">
@@ -717,14 +806,23 @@
           <t>50-75</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="3" t="n">
         <v>230.76</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>217.89</v>
-      </c>
-      <c r="D5" s="5" t="n">
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>196.89</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F5" s="3" t="n">
         <v>180.24</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -733,20 +831,29 @@
           <t>75-100</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="3" t="n">
         <v>317.09</v>
       </c>
-      <c r="C6" s="5" t="n">
-        <v>299.99</v>
-      </c>
-      <c r="D6" s="5" t="n">
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>270.23</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>29.76</v>
+      </c>
+      <c r="F6" s="3" t="n">
         <v>247.83</v>
       </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Standard decks. CK calibrated to real carts. TCG shipping: Direct free &gt;$50, other sellers blended $5/$1.49, ~$30 full deck. ManaPool = public retail. 2026-07 prices.</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Standard decks. CK calibrated to real carts. TCG shipping: Direct free &gt;$50, other sellers blended $5/$1.49 (~$30 full deck). ManaPool = public retail. 2026-07.</t>
         </is>
       </c>
     </row>

</xml_diff>